<commit_message>
Updated germination_data.csv for most recent numbers
</commit_message>
<xml_diff>
--- a/analyses/inputs/germination_data_messy.xlsx
+++ b/analyses/inputs/germination_data_messy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nolanmeier/git/morasoilinoculation/analyses/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{67E88531-6D88-A54E-BF29-D247EC239329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5E3268C-95CB-0E46-8A22-27B432BD90A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4420" yWindow="680" windowWidth="24980" windowHeight="17260" xr2:uid="{8DD11EFF-0136-EA44-86B7-80FED636BE50}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="94">
   <si>
     <t>seed_species</t>
   </si>
@@ -164,9 +164,6 @@
   </si>
   <si>
     <t>doy296: mold on soil; doy303: no obvious signs of mold on soil; doy328: previously dead germinant is still quite green, so marking as alive this week</t>
-  </si>
-  <si>
-    <t>doy296: mold on soil; doy303: no obvious signs of mold on soil; doy310: germinant not dead but unhealthy; doy328: dead germinant appears to still be alive, very green</t>
   </si>
   <si>
     <t>doy328: could not find dead germinant, but assumed its there since all 5 look healthy</t>
@@ -338,6 +335,12 @@
   <si>
     <t>doy63: previous measurements invalid, 5 alive, 2 dead, one hald dead</t>
   </si>
+  <si>
+    <t>doy296: mold on soil; doy 358: green moss?;doy63: previous measurements invalid, 8 alive 1 dead</t>
+  </si>
+  <si>
+    <t>doy296: mold on soil; doy303: no obvious signs of mold on soil; doy310: germinant not dead but unhealthy; doy328: dead germinant appears to still be alive, very green; doy63:previous measurements invalid, 9 alive 1 half dead</t>
+  </si>
 </sst>
 </file>
 
@@ -365,7 +368,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -375,6 +378,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC0E6F5"/>
+        <bgColor rgb="FFC0E6F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFC0E6F5"/>
       </patternFill>
     </fill>
@@ -402,10 +417,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -425,23 +443,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}" name="Table1" displayName="Table1" ref="B2:BI213" totalsRowShown="0">
-  <autoFilter ref="B2:BI213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="THPL"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="1">
-      <filters>
-        <filter val="PSME"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="2">
-      <filters>
-        <filter val="25"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B2:BI213" xr:uid="{7BC992C1-6373-AD4D-8EE4-164E75FC3419}"/>
   <tableColumns count="60">
     <tableColumn id="1" xr3:uid="{1199D7AD-452C-9D4F-9453-306631F01BCC}" name="soil_species"/>
     <tableColumn id="2" xr3:uid="{11F49906-5A0D-4E4F-BA5C-F91CB62A2174}" name="seed_species"/>
@@ -825,7 +827,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68F8197-A530-A948-B005-AEDF71CF4B66}">
-  <dimension ref="B2:BI213"/>
+  <dimension ref="B2:BI212"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -910,112 +912,112 @@
         <v>40</v>
       </c>
       <c r="AA2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB2" t="s">
         <v>44</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AC2" t="s">
         <v>45</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AD2" t="s">
         <v>46</v>
       </c>
-      <c r="AD2" t="s">
-        <v>47</v>
-      </c>
       <c r="AE2" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF2" t="s">
         <v>49</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AG2" t="s">
         <v>50</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AH2" t="s">
         <v>51</v>
       </c>
-      <c r="AH2" t="s">
+      <c r="AI2" t="s">
         <v>52</v>
       </c>
-      <c r="AI2" t="s">
+      <c r="AJ2" t="s">
         <v>53</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AK2" t="s">
         <v>54</v>
       </c>
-      <c r="AK2" t="s">
+      <c r="AL2" t="s">
         <v>55</v>
       </c>
-      <c r="AL2" t="s">
+      <c r="AM2" t="s">
+        <v>57</v>
+      </c>
+      <c r="AN2" t="s">
         <v>56</v>
       </c>
-      <c r="AM2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>57</v>
-      </c>
       <c r="AO2" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP2" t="s">
         <v>69</v>
       </c>
-      <c r="AP2" t="s">
+      <c r="AQ2" t="s">
         <v>70</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="AR2" t="s">
         <v>71</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="AS2" t="s">
         <v>72</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AT2" t="s">
         <v>73</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="AU2" t="s">
         <v>74</v>
       </c>
-      <c r="AU2" t="s">
+      <c r="AV2" t="s">
         <v>75</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="AW2" t="s">
         <v>76</v>
       </c>
-      <c r="AW2" t="s">
+      <c r="AX2" t="s">
         <v>77</v>
       </c>
-      <c r="AX2" t="s">
+      <c r="AY2" t="s">
         <v>78</v>
       </c>
-      <c r="AY2" t="s">
+      <c r="AZ2" t="s">
         <v>79</v>
       </c>
-      <c r="AZ2" t="s">
+      <c r="BA2" t="s">
         <v>80</v>
       </c>
-      <c r="BA2" t="s">
+      <c r="BB2" t="s">
         <v>81</v>
       </c>
-      <c r="BB2" t="s">
+      <c r="BC2" t="s">
         <v>82</v>
       </c>
-      <c r="BC2" t="s">
+      <c r="BD2" t="s">
         <v>83</v>
       </c>
-      <c r="BD2" t="s">
+      <c r="BE2" t="s">
         <v>84</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BF2" t="s">
         <v>85</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BG2" t="s">
         <v>86</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BH2" t="s">
         <v>87</v>
       </c>
-      <c r="BH2" t="s">
+      <c r="BI2" t="s">
         <v>88</v>
       </c>
-      <c r="BI2" t="s">
-        <v>89</v>
-      </c>
     </row>
-    <row r="3" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -1161,7 +1163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1175,7 +1177,7 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -1250,7 +1252,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1396,7 +1398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -1485,7 +1487,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -1598,7 +1600,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>1</v>
       </c>
@@ -1738,7 +1740,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>1</v>
       </c>
@@ -1884,7 +1886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -1976,7 +1978,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -2116,7 +2118,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>4</v>
       </c>
@@ -2265,7 +2267,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -2387,7 +2389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -2497,7 +2499,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
         <v>3</v>
       </c>
@@ -2512,7 +2514,7 @@
         <v>2</v>
       </c>
       <c r="F15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M15">
         <v>2</v>
@@ -2623,7 +2625,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
         <v>3</v>
       </c>
@@ -2734,7 +2736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>3</v>
       </c>
@@ -2869,7 +2871,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>3</v>
       </c>
@@ -2953,7 +2955,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -2968,7 +2970,7 @@
         <v>2</v>
       </c>
       <c r="F19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Q19">
         <v>4</v>
@@ -3091,7 +3093,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>1</v>
       </c>
@@ -3202,7 +3204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
         <v>1</v>
       </c>
@@ -3318,7 +3320,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
         <v>1</v>
       </c>
@@ -3408,7 +3410,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
         <v>4</v>
       </c>
@@ -3534,7 +3536,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
         <v>4</v>
       </c>
@@ -3549,7 +3551,7 @@
         <v>2</v>
       </c>
       <c r="F24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M24">
         <v>1</v>
@@ -3651,7 +3653,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
         <v>4</v>
       </c>
@@ -3738,7 +3740,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -3903,13 +3905,13 @@
         <v>6</v>
       </c>
       <c r="BH26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BI26">
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
         <v>3</v>
       </c>
@@ -3924,7 +3926,7 @@
         <v>3</v>
       </c>
       <c r="F27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M27">
         <v>4</v>
@@ -4008,7 +4010,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
         <v>3</v>
       </c>
@@ -4158,127 +4160,127 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B29" t="s">
-        <v>3</v>
-      </c>
-      <c r="C29" t="s">
-        <v>1</v>
-      </c>
-      <c r="D29">
+    <row r="29" spans="2:61" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B29" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D29" s="3">
         <v>10</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="5">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="F29" t="s">
-        <v>90</v>
-      </c>
-      <c r="M29">
-        <v>1</v>
-      </c>
-      <c r="O29">
-        <v>2</v>
-      </c>
-      <c r="Q29">
-        <v>3</v>
-      </c>
-      <c r="S29">
-        <v>4</v>
-      </c>
-      <c r="U29">
-        <v>4</v>
-      </c>
-      <c r="W29">
-        <v>4</v>
-      </c>
-      <c r="Y29">
-        <v>4</v>
-      </c>
-      <c r="AA29">
-        <v>4</v>
-      </c>
-      <c r="AC29">
-        <v>4</v>
-      </c>
-      <c r="AE29">
-        <v>4</v>
-      </c>
-      <c r="AG29">
-        <v>4</v>
-      </c>
-      <c r="AI29">
-        <v>4</v>
-      </c>
-      <c r="AK29">
-        <v>4</v>
-      </c>
-      <c r="AM29">
-        <v>4</v>
-      </c>
-      <c r="AO29">
-        <v>4</v>
-      </c>
-      <c r="AQ29">
-        <v>3</v>
-      </c>
-      <c r="AR29">
-        <v>1</v>
-      </c>
-      <c r="AS29">
-        <v>3</v>
-      </c>
-      <c r="AT29">
-        <v>1</v>
-      </c>
-      <c r="AU29">
-        <v>3</v>
-      </c>
-      <c r="AV29">
-        <v>1</v>
-      </c>
-      <c r="AW29">
-        <v>3</v>
-      </c>
-      <c r="AX29">
-        <v>1</v>
-      </c>
-      <c r="AY29">
-        <v>3</v>
-      </c>
-      <c r="AZ29">
-        <v>1</v>
-      </c>
-      <c r="BA29">
-        <v>3</v>
-      </c>
-      <c r="BB29">
-        <v>1</v>
-      </c>
-      <c r="BC29">
-        <v>3</v>
-      </c>
-      <c r="BD29">
-        <v>1</v>
-      </c>
-      <c r="BE29">
-        <v>3</v>
-      </c>
-      <c r="BF29">
-        <v>1</v>
-      </c>
-      <c r="BG29">
-        <v>4</v>
-      </c>
-      <c r="BH29">
+      <c r="F29" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="M29" s="3">
+        <v>1</v>
+      </c>
+      <c r="O29" s="3">
+        <v>2</v>
+      </c>
+      <c r="Q29" s="3">
+        <v>3</v>
+      </c>
+      <c r="S29" s="3">
+        <v>4</v>
+      </c>
+      <c r="U29" s="3">
+        <v>4</v>
+      </c>
+      <c r="W29" s="3">
+        <v>4</v>
+      </c>
+      <c r="Y29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AA29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AC29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AE29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AG29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AI29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AK29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AM29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AO29" s="3">
+        <v>4</v>
+      </c>
+      <c r="AQ29" s="3">
+        <v>3</v>
+      </c>
+      <c r="AR29" s="3">
+        <v>1</v>
+      </c>
+      <c r="AS29" s="3">
+        <v>3</v>
+      </c>
+      <c r="AT29" s="3">
+        <v>1</v>
+      </c>
+      <c r="AU29" s="3">
+        <v>3</v>
+      </c>
+      <c r="AV29" s="3">
+        <v>1</v>
+      </c>
+      <c r="AW29" s="3">
+        <v>3</v>
+      </c>
+      <c r="AX29" s="3">
+        <v>1</v>
+      </c>
+      <c r="AY29" s="3">
+        <v>3</v>
+      </c>
+      <c r="AZ29" s="3">
+        <v>1</v>
+      </c>
+      <c r="BA29" s="3">
+        <v>3</v>
+      </c>
+      <c r="BB29" s="3">
+        <v>1</v>
+      </c>
+      <c r="BC29" s="3">
+        <v>3</v>
+      </c>
+      <c r="BD29" s="3">
+        <v>1</v>
+      </c>
+      <c r="BE29" s="3">
+        <v>3</v>
+      </c>
+      <c r="BF29" s="3">
+        <v>1</v>
+      </c>
+      <c r="BG29" s="3">
+        <v>4</v>
+      </c>
+      <c r="BH29" s="3">
         <v>0</v>
       </c>
-      <c r="BI29">
+      <c r="BI29" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
         <v>3</v>
       </c>
@@ -4371,7 +4373,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
         <v>1</v>
       </c>
@@ -4515,7 +4517,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
         <v>1</v>
       </c>
@@ -4623,7 +4625,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
         <v>1</v>
       </c>
@@ -4725,7 +4727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
         <v>1</v>
       </c>
@@ -4842,7 +4844,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
         <v>4</v>
       </c>
@@ -4857,7 +4859,7 @@
         <v>3</v>
       </c>
       <c r="F35" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O35">
         <v>2</v>
@@ -4965,7 +4967,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
         <v>4</v>
       </c>
@@ -4980,7 +4982,7 @@
         <v>3</v>
       </c>
       <c r="F36" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="O36">
         <v>1</v>
@@ -5072,11 +5074,14 @@
       <c r="BG36">
         <v>8</v>
       </c>
+      <c r="BH36">
+        <v>1</v>
+      </c>
       <c r="BI36">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
         <v>4</v>
       </c>
@@ -5163,7 +5168,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
         <v>4</v>
       </c>
@@ -5325,7 +5330,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
         <v>3</v>
       </c>
@@ -5469,7 +5474,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
         <v>3</v>
       </c>
@@ -5484,7 +5489,7 @@
         <v>4</v>
       </c>
       <c r="F40" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M40">
         <v>1</v>
@@ -5625,7 +5630,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
         <v>3</v>
       </c>
@@ -5748,7 +5753,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
         <v>3</v>
       </c>
@@ -5844,7 +5849,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
         <v>1</v>
       </c>
@@ -5985,7 +5990,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="44" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
         <v>1</v>
       </c>
@@ -6066,7 +6071,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -6237,7 +6242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
         <v>1</v>
       </c>
@@ -6330,7 +6335,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
         <v>4</v>
       </c>
@@ -6345,7 +6350,7 @@
         <v>4</v>
       </c>
       <c r="F47" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O47">
         <v>1</v>
@@ -6429,7 +6434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
         <v>4</v>
       </c>
@@ -6444,7 +6449,7 @@
         <v>4</v>
       </c>
       <c r="F48" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M48">
         <v>1</v>
@@ -6585,7 +6590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
         <v>4</v>
       </c>
@@ -6672,7 +6677,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
         <v>4</v>
       </c>
@@ -6840,7 +6845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
         <v>3</v>
       </c>
@@ -6855,7 +6860,7 @@
         <v>5</v>
       </c>
       <c r="F51" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M51">
         <v>0</v>
@@ -6984,7 +6989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
         <v>3</v>
       </c>
@@ -7071,7 +7076,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
         <v>3</v>
       </c>
@@ -7203,7 +7208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B54" t="s">
         <v>3</v>
       </c>
@@ -7293,7 +7298,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B55" t="s">
         <v>1</v>
       </c>
@@ -7419,7 +7424,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B56" t="s">
         <v>1</v>
       </c>
@@ -7500,7 +7505,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B57" t="s">
         <v>1</v>
       </c>
@@ -7587,7 +7592,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B58" t="s">
         <v>1</v>
       </c>
@@ -7680,7 +7685,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B59" t="s">
         <v>4</v>
       </c>
@@ -7764,7 +7769,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="60" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B60" t="s">
         <v>4</v>
       </c>
@@ -7890,7 +7895,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B61" t="s">
         <v>4</v>
       </c>
@@ -7980,7 +7985,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B62" t="s">
         <v>4</v>
       </c>
@@ -7995,7 +8000,7 @@
         <v>5</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K62">
         <v>2</v>
@@ -8136,7 +8141,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="63" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B63" t="s">
         <v>3</v>
       </c>
@@ -8151,7 +8156,7 @@
         <v>6</v>
       </c>
       <c r="F63" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M63">
         <v>1</v>
@@ -8274,7 +8279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B64" t="s">
         <v>3</v>
       </c>
@@ -8382,7 +8387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B65" t="s">
         <v>3</v>
       </c>
@@ -8493,7 +8498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B66" t="s">
         <v>3</v>
       </c>
@@ -8580,7 +8585,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B67" t="s">
         <v>1</v>
       </c>
@@ -8727,7 +8732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B68" t="s">
         <v>1</v>
       </c>
@@ -8808,7 +8813,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="69" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B69" t="s">
         <v>1</v>
       </c>
@@ -8895,7 +8900,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="70" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B70" t="s">
         <v>1</v>
       </c>
@@ -8991,7 +8996,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="71" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B71" t="s">
         <v>4</v>
       </c>
@@ -9006,7 +9011,7 @@
         <v>6</v>
       </c>
       <c r="F71" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O71">
         <v>4</v>
@@ -9117,7 +9122,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B72" t="s">
         <v>4</v>
       </c>
@@ -9132,7 +9137,7 @@
         <v>6</v>
       </c>
       <c r="F72" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O72">
         <v>2</v>
@@ -9252,7 +9257,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B73" t="s">
         <v>4</v>
       </c>
@@ -9339,7 +9344,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="74" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B74" t="s">
         <v>4</v>
       </c>
@@ -9435,7 +9440,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B75" t="s">
         <v>3</v>
       </c>
@@ -9450,7 +9455,7 @@
         <v>7</v>
       </c>
       <c r="F75" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M75">
         <v>1</v>
@@ -9555,7 +9560,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B76" t="s">
         <v>3</v>
       </c>
@@ -9570,7 +9575,7 @@
         <v>7</v>
       </c>
       <c r="F76" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M76">
         <v>1</v>
@@ -9708,7 +9713,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B77" t="s">
         <v>3</v>
       </c>
@@ -9813,7 +9818,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B78" t="s">
         <v>3</v>
       </c>
@@ -9903,7 +9908,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="79" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B79" t="s">
         <v>1</v>
       </c>
@@ -10050,7 +10055,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="80" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B80" t="s">
         <v>1</v>
       </c>
@@ -10167,7 +10172,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B81" t="s">
         <v>1</v>
       </c>
@@ -10296,7 +10301,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B82" t="s">
         <v>1</v>
       </c>
@@ -10443,7 +10448,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B83" t="s">
         <v>4</v>
       </c>
@@ -10458,7 +10463,7 @@
         <v>7</v>
       </c>
       <c r="F83" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O83">
         <v>2</v>
@@ -10590,7 +10595,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="84" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B84" t="s">
         <v>4</v>
       </c>
@@ -10605,7 +10610,7 @@
         <v>7</v>
       </c>
       <c r="F84" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O84">
         <v>2</v>
@@ -10737,7 +10742,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="85" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B85" t="s">
         <v>4</v>
       </c>
@@ -10752,7 +10757,7 @@
         <v>7</v>
       </c>
       <c r="F85" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M85">
         <v>3</v>
@@ -10881,7 +10886,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="86" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B86" t="s">
         <v>4</v>
       </c>
@@ -11007,7 +11012,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B87" t="s">
         <v>3</v>
       </c>
@@ -11022,7 +11027,7 @@
         <v>8</v>
       </c>
       <c r="F87" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M87">
         <v>2</v>
@@ -11157,7 +11162,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="88" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B88" t="s">
         <v>3</v>
       </c>
@@ -11172,7 +11177,7 @@
         <v>8</v>
       </c>
       <c r="F88" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M88">
         <v>0</v>
@@ -11292,121 +11297,121 @@
         <v>3</v>
       </c>
     </row>
-    <row r="89" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B89" t="s">
-        <v>3</v>
-      </c>
-      <c r="C89" t="s">
-        <v>1</v>
-      </c>
-      <c r="D89">
+    <row r="89" spans="2:61" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B89" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D89" s="3">
         <v>10</v>
       </c>
-      <c r="E89" s="2">
+      <c r="E89" s="5">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="F89" t="s">
-        <v>91</v>
-      </c>
-      <c r="K89">
-        <v>1</v>
-      </c>
-      <c r="M89">
-        <v>4</v>
-      </c>
-      <c r="O89">
-        <v>4</v>
-      </c>
-      <c r="Q89">
-        <v>5</v>
-      </c>
-      <c r="S89">
-        <v>5</v>
-      </c>
-      <c r="U89">
-        <v>5</v>
-      </c>
-      <c r="W89">
-        <v>5</v>
-      </c>
-      <c r="Y89">
-        <v>5</v>
-      </c>
-      <c r="AA89">
-        <v>5</v>
-      </c>
-      <c r="AC89">
-        <v>5</v>
-      </c>
-      <c r="AE89">
-        <v>5</v>
-      </c>
-      <c r="AG89">
-        <v>5</v>
-      </c>
-      <c r="AI89">
-        <v>5</v>
-      </c>
-      <c r="AK89">
-        <v>5</v>
-      </c>
-      <c r="AM89">
-        <v>5</v>
-      </c>
-      <c r="AO89">
-        <v>5</v>
-      </c>
-      <c r="AQ89">
-        <v>5</v>
-      </c>
-      <c r="AS89">
-        <v>4</v>
-      </c>
-      <c r="AT89">
-        <v>1</v>
-      </c>
-      <c r="AU89">
-        <v>4</v>
-      </c>
-      <c r="AV89">
-        <v>1</v>
-      </c>
-      <c r="AW89">
-        <v>3</v>
-      </c>
-      <c r="AX89">
-        <v>2</v>
-      </c>
-      <c r="AY89">
-        <v>3</v>
-      </c>
-      <c r="AZ89">
-        <v>2</v>
-      </c>
-      <c r="BA89">
-        <v>3</v>
-      </c>
-      <c r="BB89">
-        <v>2</v>
-      </c>
-      <c r="BC89">
-        <v>3</v>
-      </c>
-      <c r="BD89">
-        <v>2</v>
-      </c>
-      <c r="BE89">
-        <v>3</v>
-      </c>
-      <c r="BF89">
-        <v>2</v>
-      </c>
-      <c r="BG89">
+      <c r="F89" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="K89" s="3">
+        <v>1</v>
+      </c>
+      <c r="M89" s="3">
+        <v>4</v>
+      </c>
+      <c r="O89" s="3">
+        <v>4</v>
+      </c>
+      <c r="Q89" s="3">
+        <v>5</v>
+      </c>
+      <c r="S89" s="3">
+        <v>5</v>
+      </c>
+      <c r="U89" s="3">
+        <v>5</v>
+      </c>
+      <c r="W89" s="3">
+        <v>5</v>
+      </c>
+      <c r="Y89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AA89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AC89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AE89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AG89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AI89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AK89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AM89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AO89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AQ89" s="3">
+        <v>5</v>
+      </c>
+      <c r="AS89" s="3">
+        <v>4</v>
+      </c>
+      <c r="AT89" s="3">
+        <v>1</v>
+      </c>
+      <c r="AU89" s="3">
+        <v>4</v>
+      </c>
+      <c r="AV89" s="3">
+        <v>1</v>
+      </c>
+      <c r="AW89" s="3">
+        <v>3</v>
+      </c>
+      <c r="AX89" s="3">
+        <v>2</v>
+      </c>
+      <c r="AY89" s="3">
+        <v>3</v>
+      </c>
+      <c r="AZ89" s="3">
+        <v>2</v>
+      </c>
+      <c r="BA89" s="3">
+        <v>3</v>
+      </c>
+      <c r="BB89" s="3">
+        <v>2</v>
+      </c>
+      <c r="BC89" s="3">
+        <v>3</v>
+      </c>
+      <c r="BD89" s="3">
+        <v>2</v>
+      </c>
+      <c r="BE89" s="3">
+        <v>3</v>
+      </c>
+      <c r="BF89" s="3">
+        <v>2</v>
+      </c>
+      <c r="BG89" s="3">
         <v>5</v>
       </c>
     </row>
-    <row r="90" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B90" t="s">
         <v>3</v>
       </c>
@@ -11496,7 +11501,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="91" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B91" t="s">
         <v>1</v>
       </c>
@@ -11643,133 +11648,136 @@
         <v>2</v>
       </c>
     </row>
-    <row r="92" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B92" t="s">
-        <v>1</v>
-      </c>
-      <c r="C92" t="s">
-        <v>3</v>
-      </c>
-      <c r="D92">
+    <row r="92" spans="2:61" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B92" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D92" s="3">
         <v>0</v>
       </c>
-      <c r="E92" s="1">
+      <c r="E92" s="4">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="F92" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q92">
+      <c r="F92" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q92" s="3">
         <v>0</v>
       </c>
-      <c r="S92">
-        <v>1</v>
-      </c>
-      <c r="U92">
-        <v>2</v>
-      </c>
-      <c r="W92">
-        <v>4</v>
-      </c>
-      <c r="Y92">
-        <v>4</v>
-      </c>
-      <c r="AA92">
-        <v>4</v>
-      </c>
-      <c r="AC92">
-        <v>5</v>
-      </c>
-      <c r="AE92">
-        <v>6</v>
-      </c>
-      <c r="AG92">
-        <v>5</v>
-      </c>
-      <c r="AH92">
-        <v>1</v>
-      </c>
-      <c r="AI92">
-        <v>5</v>
-      </c>
-      <c r="AJ92">
-        <v>2</v>
-      </c>
-      <c r="AK92">
-        <v>5</v>
-      </c>
-      <c r="AL92">
-        <v>2</v>
-      </c>
-      <c r="AM92">
-        <v>5</v>
-      </c>
-      <c r="AN92">
-        <v>2</v>
-      </c>
-      <c r="AO92">
-        <v>5</v>
-      </c>
-      <c r="AP92">
-        <v>2</v>
-      </c>
-      <c r="AQ92">
-        <v>5</v>
-      </c>
-      <c r="AR92">
-        <v>2</v>
-      </c>
-      <c r="AS92">
-        <v>5</v>
-      </c>
-      <c r="AT92">
-        <v>2</v>
-      </c>
-      <c r="AU92">
-        <v>5</v>
-      </c>
-      <c r="AV92">
-        <v>2</v>
-      </c>
-      <c r="AW92">
-        <v>5</v>
-      </c>
-      <c r="AX92">
-        <v>2</v>
-      </c>
-      <c r="AY92">
-        <v>5</v>
-      </c>
-      <c r="AZ92">
-        <v>2</v>
-      </c>
-      <c r="BA92">
-        <v>5</v>
-      </c>
-      <c r="BB92">
-        <v>2</v>
-      </c>
-      <c r="BC92">
-        <v>4</v>
-      </c>
-      <c r="BD92">
-        <v>3</v>
-      </c>
-      <c r="BE92">
-        <v>4</v>
-      </c>
-      <c r="BF92">
-        <v>3</v>
-      </c>
-      <c r="BG92">
-        <v>5</v>
-      </c>
-      <c r="BH92">
-        <v>2</v>
+      <c r="S92" s="3">
+        <v>1</v>
+      </c>
+      <c r="U92" s="3">
+        <v>2</v>
+      </c>
+      <c r="W92" s="3">
+        <v>4</v>
+      </c>
+      <c r="Y92" s="3">
+        <v>4</v>
+      </c>
+      <c r="AA92" s="3">
+        <v>4</v>
+      </c>
+      <c r="AC92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AE92" s="3">
+        <v>6</v>
+      </c>
+      <c r="AG92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AH92" s="3">
+        <v>1</v>
+      </c>
+      <c r="AI92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AJ92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AK92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AL92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AM92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AN92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AO92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AP92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AQ92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AR92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AS92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AT92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AU92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AV92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AW92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AX92" s="3">
+        <v>2</v>
+      </c>
+      <c r="AY92" s="3">
+        <v>5</v>
+      </c>
+      <c r="AZ92" s="3">
+        <v>2</v>
+      </c>
+      <c r="BA92" s="3">
+        <v>5</v>
+      </c>
+      <c r="BB92" s="3">
+        <v>2</v>
+      </c>
+      <c r="BC92" s="3">
+        <v>4</v>
+      </c>
+      <c r="BD92" s="3">
+        <v>3</v>
+      </c>
+      <c r="BE92" s="3">
+        <v>4</v>
+      </c>
+      <c r="BF92" s="3">
+        <v>3</v>
+      </c>
+      <c r="BG92" s="3">
+        <v>5</v>
+      </c>
+      <c r="BH92" s="3">
+        <v>2</v>
+      </c>
+      <c r="BI92" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="93" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B93" t="s">
         <v>1</v>
       </c>
@@ -11868,7 +11876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B94" t="s">
         <v>1</v>
       </c>
@@ -11961,7 +11969,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="95" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B95" t="s">
         <v>4</v>
       </c>
@@ -11976,7 +11984,7 @@
         <v>8</v>
       </c>
       <c r="F95" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O95">
         <v>2</v>
@@ -12066,7 +12074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B96" t="s">
         <v>4</v>
       </c>
@@ -12081,7 +12089,7 @@
         <v>8</v>
       </c>
       <c r="F96" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O96">
         <v>1</v>
@@ -12195,7 +12203,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="97" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B97" t="s">
         <v>4</v>
       </c>
@@ -12285,7 +12293,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="98" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B98" t="s">
         <v>4</v>
       </c>
@@ -12414,7 +12422,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="99" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B99" t="s">
         <v>3</v>
       </c>
@@ -12498,7 +12506,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="100" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B100" t="s">
         <v>3</v>
       </c>
@@ -12585,7 +12593,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="101" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B101" t="s">
         <v>3</v>
       </c>
@@ -12600,7 +12608,7 @@
         <v>9</v>
       </c>
       <c r="F101" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M101">
         <v>1</v>
@@ -12702,7 +12710,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="102" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B102" t="s">
         <v>3</v>
       </c>
@@ -12792,7 +12800,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="103" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B103" t="s">
         <v>1</v>
       </c>
@@ -12807,7 +12815,7 @@
         <v>9</v>
       </c>
       <c r="F103" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Q103">
         <v>1</v>
@@ -12930,7 +12938,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="104" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B104" t="s">
         <v>1</v>
       </c>
@@ -13044,7 +13052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B105" t="s">
         <v>1</v>
       </c>
@@ -13167,7 +13175,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B106" t="s">
         <v>1</v>
       </c>
@@ -13302,7 +13310,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="107" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B107" t="s">
         <v>4</v>
       </c>
@@ -13437,7 +13445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B108" t="s">
         <v>4</v>
       </c>
@@ -13539,7 +13547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B109" t="s">
         <v>4</v>
       </c>
@@ -13665,7 +13673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B110" t="s">
         <v>4</v>
       </c>
@@ -13680,7 +13688,7 @@
         <v>9</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>42</v>
+        <v>93</v>
       </c>
       <c r="K110">
         <v>4</v>
@@ -13794,7 +13802,7 @@
         <v>1</v>
       </c>
       <c r="BG110">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BH110">
         <v>0</v>
@@ -13803,7 +13811,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B111" t="s">
         <v>3</v>
       </c>
@@ -13911,7 +13919,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="112" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B112" t="s">
         <v>3</v>
       </c>
@@ -14040,7 +14048,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="113" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B113" t="s">
         <v>3</v>
       </c>
@@ -14184,7 +14192,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="114" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B114" t="s">
         <v>3</v>
       </c>
@@ -14274,7 +14282,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="115" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B115" t="s">
         <v>1</v>
       </c>
@@ -14289,7 +14297,7 @@
         <v>10</v>
       </c>
       <c r="F115" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="O115">
         <v>2</v>
@@ -14421,7 +14429,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="116" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B116" t="s">
         <v>1</v>
       </c>
@@ -14535,7 +14543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B117" t="s">
         <v>1</v>
       </c>
@@ -14661,7 +14669,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B118" t="s">
         <v>1</v>
       </c>
@@ -14755,7 +14763,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B119" t="s">
         <v>4</v>
       </c>
@@ -14839,7 +14847,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="120" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B120" t="s">
         <v>4</v>
       </c>
@@ -14926,7 +14934,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="121" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B121" t="s">
         <v>4</v>
       </c>
@@ -14941,7 +14949,7 @@
         <v>10</v>
       </c>
       <c r="F121" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M121">
         <v>3</v>
@@ -15016,7 +15024,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="122" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B122" t="s">
         <v>4</v>
       </c>
@@ -15109,7 +15117,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="123" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B123" t="s">
         <v>3</v>
       </c>
@@ -15235,7 +15243,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="124" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B124" t="s">
         <v>3</v>
       </c>
@@ -15388,7 +15396,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="125" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B125" t="s">
         <v>3</v>
       </c>
@@ -15403,7 +15411,7 @@
         <v>11</v>
       </c>
       <c r="F125" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="M125">
         <v>2</v>
@@ -15541,7 +15549,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="126" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B126" t="s">
         <v>3</v>
       </c>
@@ -15673,7 +15681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B127" t="s">
         <v>1</v>
       </c>
@@ -15802,7 +15810,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="128" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B128" t="s">
         <v>1</v>
       </c>
@@ -15883,7 +15891,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="129" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B129" t="s">
         <v>1</v>
       </c>
@@ -16015,7 +16023,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B130" t="s">
         <v>1</v>
       </c>
@@ -16108,7 +16116,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="131" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B131" t="s">
         <v>4</v>
       </c>
@@ -16123,7 +16131,7 @@
         <v>11</v>
       </c>
       <c r="F131" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Q131">
         <v>2</v>
@@ -16231,7 +16239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B132" t="s">
         <v>4</v>
       </c>
@@ -16315,7 +16323,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="133" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B133" t="s">
         <v>4</v>
       </c>
@@ -16414,7 +16422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B134" t="s">
         <v>4</v>
       </c>
@@ -16510,7 +16518,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B135" t="s">
         <v>3</v>
       </c>
@@ -16612,7 +16620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B136" t="s">
         <v>3</v>
       </c>
@@ -16723,7 +16731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B137" t="s">
         <v>3</v>
       </c>
@@ -16840,7 +16848,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="138" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B138" t="s">
         <v>3</v>
       </c>
@@ -16975,7 +16983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B139" t="s">
         <v>1</v>
       </c>
@@ -17092,7 +17100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B140" t="s">
         <v>1</v>
       </c>
@@ -17173,7 +17181,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="141" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B141" t="s">
         <v>1</v>
       </c>
@@ -17329,7 +17337,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="142" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B142" t="s">
         <v>1</v>
       </c>
@@ -17482,7 +17490,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="143" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B143" t="s">
         <v>4</v>
       </c>
@@ -17581,7 +17589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B144" t="s">
         <v>4</v>
       </c>
@@ -17665,7 +17673,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="145" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B145" t="s">
         <v>4</v>
       </c>
@@ -17755,7 +17763,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="146" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B146" t="s">
         <v>4</v>
       </c>
@@ -17893,7 +17901,7 @@
         <v>2</v>
       </c>
       <c r="BG146">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BH146">
         <v>1</v>
@@ -17902,7 +17910,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B147" t="s">
         <v>3</v>
       </c>
@@ -17917,7 +17925,7 @@
         <v>13</v>
       </c>
       <c r="F147" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O147">
         <v>0</v>
@@ -18040,7 +18048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B148" t="s">
         <v>3</v>
       </c>
@@ -18127,7 +18135,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="149" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B149" t="s">
         <v>3</v>
       </c>
@@ -18256,7 +18264,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="150" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B150" t="s">
         <v>3</v>
       </c>
@@ -18406,7 +18414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B151" t="s">
         <v>1</v>
       </c>
@@ -18421,7 +18429,7 @@
         <v>13</v>
       </c>
       <c r="F151" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Q151">
         <v>1</v>
@@ -18508,7 +18516,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="152" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B152" t="s">
         <v>1</v>
       </c>
@@ -18589,7 +18597,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="153" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B153" t="s">
         <v>1</v>
       </c>
@@ -18703,7 +18711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B154" t="s">
         <v>1</v>
       </c>
@@ -18718,7 +18726,7 @@
         <v>13</v>
       </c>
       <c r="F154" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K154">
         <v>0</v>
@@ -18865,7 +18873,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B155" t="s">
         <v>4</v>
       </c>
@@ -18991,7 +18999,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="156" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B156" t="s">
         <v>4</v>
       </c>
@@ -19078,7 +19086,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="157" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B157" t="s">
         <v>4</v>
       </c>
@@ -19093,7 +19101,7 @@
         <v>13</v>
       </c>
       <c r="F157" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M157">
         <v>3</v>
@@ -19168,7 +19176,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="158" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B158" t="s">
         <v>4</v>
       </c>
@@ -19264,7 +19272,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="159" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B159" t="s">
         <v>3</v>
       </c>
@@ -19393,7 +19401,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B160" t="s">
         <v>3</v>
       </c>
@@ -19480,7 +19488,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="161" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B161" t="s">
         <v>3</v>
       </c>
@@ -19633,7 +19641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B162" t="s">
         <v>3</v>
       </c>
@@ -19723,7 +19731,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="163" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B163" t="s">
         <v>1</v>
       </c>
@@ -19846,7 +19854,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B164" t="s">
         <v>1</v>
       </c>
@@ -19927,7 +19935,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="165" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B165" t="s">
         <v>1</v>
       </c>
@@ -20050,7 +20058,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="166" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B166" t="s">
         <v>1</v>
       </c>
@@ -20182,7 +20190,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="167" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B167" t="s">
         <v>4</v>
       </c>
@@ -20293,7 +20301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B168" t="s">
         <v>4</v>
       </c>
@@ -20425,7 +20433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B169" t="s">
         <v>4</v>
       </c>
@@ -20440,7 +20448,7 @@
         <v>14</v>
       </c>
       <c r="F169" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M169">
         <v>2</v>
@@ -20515,7 +20523,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="170" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B170" t="s">
         <v>4</v>
       </c>
@@ -20605,7 +20613,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="171" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B171" t="s">
         <v>3</v>
       </c>
@@ -20620,7 +20628,7 @@
         <v>15</v>
       </c>
       <c r="F171" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O171">
         <v>2</v>
@@ -20743,7 +20751,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="172" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B172" t="s">
         <v>3</v>
       </c>
@@ -20830,7 +20838,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="173" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B173" t="s">
         <v>3</v>
       </c>
@@ -20917,7 +20925,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="174" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B174" t="s">
         <v>3</v>
       </c>
@@ -21007,7 +21015,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="175" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B175" t="s">
         <v>1</v>
       </c>
@@ -21130,7 +21138,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="176" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B176" t="s">
         <v>1</v>
       </c>
@@ -21211,7 +21219,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="177" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B177" t="s">
         <v>1</v>
       </c>
@@ -21298,7 +21306,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="178" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B178" t="s">
         <v>1</v>
       </c>
@@ -21313,7 +21321,7 @@
         <v>15</v>
       </c>
       <c r="F178" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K178">
         <v>1</v>
@@ -21391,7 +21399,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="179" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B179" t="s">
         <v>4</v>
       </c>
@@ -21517,7 +21525,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="180" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B180" t="s">
         <v>4</v>
       </c>
@@ -21637,7 +21645,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="181" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B181" t="s">
         <v>4</v>
       </c>
@@ -21754,7 +21762,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="182" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B182" t="s">
         <v>4</v>
       </c>
@@ -21844,7 +21852,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="183" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B183" t="s">
         <v>3</v>
       </c>
@@ -21858,7 +21866,7 @@
         <v>1</v>
       </c>
       <c r="F183" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="O183">
         <v>0</v>
@@ -21987,7 +21995,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="184" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B184" t="s">
         <v>1</v>
       </c>
@@ -22073,7 +22081,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="185" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B185" t="s">
         <v>3</v>
       </c>
@@ -22183,13 +22191,13 @@
         <v>2</v>
       </c>
       <c r="BH185">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BI185">
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B186" t="s">
         <v>1</v>
       </c>
@@ -22308,7 +22316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B187" t="s">
         <v>4</v>
       </c>
@@ -22516,7 +22524,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="189" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B189" t="s">
         <v>3</v>
       </c>
@@ -22530,7 +22538,7 @@
         <v>2</v>
       </c>
       <c r="F189" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O189">
         <v>0</v>
@@ -22662,7 +22670,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="190" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B190" t="s">
         <v>1</v>
       </c>
@@ -22676,7 +22684,7 @@
         <v>2</v>
       </c>
       <c r="F190" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M190">
         <v>0</v>
@@ -22799,7 +22807,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="191" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B191" t="s">
         <v>3</v>
       </c>
@@ -22813,7 +22821,7 @@
         <v>2</v>
       </c>
       <c r="F191" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K191">
         <v>1</v>
@@ -22939,7 +22947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B192" t="s">
         <v>1</v>
       </c>
@@ -23061,7 +23069,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="193" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B193" t="s">
         <v>4</v>
       </c>
@@ -23323,7 +23331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B195" t="s">
         <v>3</v>
       </c>
@@ -23337,7 +23345,7 @@
         <v>3</v>
       </c>
       <c r="F195" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O195">
         <v>0</v>
@@ -23466,7 +23474,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="196" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B196" t="s">
         <v>1</v>
       </c>
@@ -23480,7 +23488,7 @@
         <v>3</v>
       </c>
       <c r="F196" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K196">
         <v>1</v>
@@ -23618,7 +23626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="197" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B197" t="s">
         <v>3</v>
       </c>
@@ -23740,7 +23748,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="198" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B198" t="s">
         <v>1</v>
       </c>
@@ -23835,7 +23843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="199" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B199" t="s">
         <v>4</v>
       </c>
@@ -23957,7 +23965,7 @@
         <v>1</v>
       </c>
       <c r="BG199">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BI199">
         <v>1</v>
@@ -24070,7 +24078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="201" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B201" t="s">
         <v>3</v>
       </c>
@@ -24084,7 +24092,7 @@
         <v>4</v>
       </c>
       <c r="F201" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O201">
         <v>0</v>
@@ -24207,7 +24215,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="202" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B202" t="s">
         <v>1</v>
       </c>
@@ -24221,7 +24229,7 @@
         <v>4</v>
       </c>
       <c r="F202" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M202">
         <v>0</v>
@@ -24350,7 +24358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="203" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B203" t="s">
         <v>3</v>
       </c>
@@ -24481,7 +24489,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B204" t="s">
         <v>1</v>
       </c>
@@ -24567,7 +24575,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="205" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B205" t="s">
         <v>4</v>
       </c>
@@ -24799,7 +24807,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="207" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B207" t="s">
         <v>3</v>
       </c>
@@ -24813,7 +24821,7 @@
         <v>5</v>
       </c>
       <c r="F207" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O207">
         <v>1</v>
@@ -24903,7 +24911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="2:61" hidden="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="2:61" x14ac:dyDescent="0.2">
       <c r="B208" t="s">
         <v>1</v>
       </c>
@@ -25040,7 +25048,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="209" spans="2:60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="2:60" x14ac:dyDescent="0.2">
       <c r="B209" t="s">
         <v>3</v>
       </c>
@@ -25054,7 +25062,7 @@
         <v>5</v>
       </c>
       <c r="F209" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M209">
         <v>1</v>
@@ -25159,7 +25167,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="210" spans="2:60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="2:60" x14ac:dyDescent="0.2">
       <c r="B210" t="s">
         <v>1</v>
       </c>
@@ -25302,7 +25310,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="2:60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="2:60" x14ac:dyDescent="0.2">
       <c r="B211" t="s">
         <v>4</v>
       </c>
@@ -25534,7 +25542,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="213" spans="2:60" hidden="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>